<commit_message>
chore(auto): checkpoint — features/cave-dossier, (root) (18 files)
Automatic commit by the checkpoint hook (.claude/hooks/auto-commit.sh).
Not a curated commit — see /wrap-up commits for session narrative.

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/features/cave-dossier/tests/fixtures/mini_sb.xlsx
+++ b/features/cave-dossier/tests/fixtures/mini_sb.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:T7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -475,6 +475,61 @@
           <t>Y HTRS</t>
         </is>
       </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Sinonimi</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Lokalitet</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Najbliže mjesto</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Duljina</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Dubina</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Napomena</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Fotografija ulaza</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Zagađenost</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Ledenica</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Godina zadnjeg istraživanja</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -518,6 +573,55 @@
       <c r="I3" t="n">
         <v>5023456</v>
       </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Testovka mala</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Testni kras</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Testno Selo</t>
+        </is>
+      </c>
+      <c r="M3" t="n">
+        <v>40</v>
+      </c>
+      <c r="N3" t="n">
+        <v>12</v>
+      </c>
+      <c r="O3" t="n">
+        <v>500</v>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>DA</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>NE</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>NE</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -556,6 +660,45 @@
       <c r="I4" t="n">
         <v>5024000.5</v>
       </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Testni kras</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Testno Selo</t>
+        </is>
+      </c>
+      <c r="M4" t="n">
+        <v>15</v>
+      </c>
+      <c r="N4" t="n">
+        <v>30</v>
+      </c>
+      <c r="O4" t="n">
+        <v>610</v>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>NE</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>NE</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>NE</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -589,6 +732,30 @@
       <c r="I5" t="n">
         <v>5025555</v>
       </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Kuk</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Gornje Testno</t>
+        </is>
+      </c>
+      <c r="M5" t="n">
+        <v>25</v>
+      </c>
+      <c r="N5" t="n">
+        <v>8</v>
+      </c>
+      <c r="O5" t="n">
+        <v>300</v>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -596,14 +763,14 @@
           <t>Đulin ponor mali</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>004</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>T-04</t>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>za istražit, 268, treba ponoviti</t>
         </is>
       </c>
     </row>
@@ -635,12 +802,12 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Ana Anić</t>
+          <t>Malez, M. (1960)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>1960</t>
         </is>
       </c>
       <c r="H7" t="n">
@@ -648,6 +815,50 @@
       </c>
       <c r="I7" t="n">
         <v>5026666</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Žedno</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Donje Testno</t>
+        </is>
+      </c>
+      <c r="M7" t="n">
+        <v>12</v>
+      </c>
+      <c r="N7" t="n">
+        <v>4</v>
+      </c>
+      <c r="O7" t="n">
+        <v>200</v>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>stari zapis</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>NE</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>NE</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>NE</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>1960</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(auto): checkpoint — features/cave-dossier, (root) (19 files)
Automatic commit by the checkpoint hook (.claude/hooks/auto-commit.sh).
Not a curated commit — see /wrap-up commits for session narrative.

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/features/cave-dossier/tests/fixtures/mini_sb.xlsx
+++ b/features/cave-dossier/tests/fixtures/mini_sb.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T7"/>
+  <dimension ref="A1:U8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -423,7 +423,7 @@
           <t>Speleo baza TEST</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>v0.0</t>
         </is>
@@ -432,432 +432,490 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>Redni broj</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>IME OBJEKTA</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Katastarski broj SUE</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>CroSpeleo unos</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Katastarski broj RH</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Broj pločice</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Autori nacrta</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Godina ili period istraživanja</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>x htrs</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Y HTRS</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Sinonimi</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>Lokalitet</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>Najbliže mjesto</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>Duljina</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>Dubina</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>Z</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>Napomena</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>Fotografija ulaza</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="S2" t="inlineStr">
         <is>
           <t>Zagađenost</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="T2" t="inlineStr">
         <is>
           <t>Ledenica</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>Godina zadnjeg istraživanja</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
         <is>
           <t>Špilja Testovka</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>001</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>1. krug</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>unesen</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>T-01</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Ana Anić</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>2015</t>
         </is>
       </c>
-      <c r="H3" t="n">
+      <c r="I3" t="n">
         <v>450123</v>
       </c>
-      <c r="I3" t="n">
+      <c r="J3" t="n">
         <v>5023456</v>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>Testovka mala</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>Testni kras</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>Testno Selo</t>
         </is>
       </c>
-      <c r="M3" t="n">
+      <c r="N3" t="n">
         <v>40</v>
       </c>
-      <c r="N3" t="n">
+      <c r="O3" t="n">
         <v>12</v>
       </c>
-      <c r="O3" t="n">
+      <c r="P3" t="n">
         <v>500</v>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t>DA</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="S3" t="inlineStr">
         <is>
           <t>NE</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="T3" t="inlineStr">
         <is>
           <t>NE</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="U3" t="inlineStr">
         <is>
           <t>2015</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="inlineStr">
         <is>
           <t>Jama Čavlić</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>002</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>1. krug</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>T-02</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Ivo Ivić; Ana Anić</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>2018-2019</t>
         </is>
       </c>
-      <c r="H4" t="n">
+      <c r="I4" t="n">
         <v>451000.5</v>
       </c>
-      <c r="I4" t="n">
+      <c r="J4" t="n">
         <v>5024000.5</v>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>Testni kras</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>Testno Selo</t>
         </is>
       </c>
-      <c r="M4" t="n">
+      <c r="N4" t="n">
         <v>15</v>
       </c>
-      <c r="N4" t="n">
+      <c r="O4" t="n">
         <v>30</v>
       </c>
-      <c r="O4" t="n">
+      <c r="P4" t="n">
         <v>610</v>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>NE</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t>NE</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
+      <c r="T4" t="inlineStr">
         <is>
           <t>NE</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>2019</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>Ponor pod Kukom</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>003</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>2. krug</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>Ivo Ivić</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>2021</t>
         </is>
       </c>
-      <c r="H5" t="n">
+      <c r="I5" t="n">
         <v>452222</v>
       </c>
-      <c r="I5" t="n">
+      <c r="J5" t="n">
         <v>5025555</v>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>Kuk</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>Gornje Testno</t>
         </is>
       </c>
-      <c r="M5" t="n">
+      <c r="N5" t="n">
         <v>25</v>
       </c>
-      <c r="N5" t="n">
+      <c r="O5" t="n">
         <v>8</v>
       </c>
-      <c r="O5" t="n">
+      <c r="P5" t="n">
         <v>300</v>
       </c>
-      <c r="T5" t="inlineStr">
+      <c r="U5" t="inlineStr">
         <is>
           <t>2021</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" t="inlineStr">
         <is>
           <t>Đulin ponor mali</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>/</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
+      <c r="Q6" t="inlineStr">
         <is>
           <t>za istražit, 268, treba ponoviti</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" t="inlineStr">
         <is>
           <t>Pećina žedna</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>005</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>2. krug</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>fali izjava</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>T-05</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>Malez, M. (1960)</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>1960</t>
         </is>
       </c>
-      <c r="H7" t="n">
+      <c r="I7" t="n">
         <v>453333</v>
       </c>
-      <c r="I7" t="n">
+      <c r="J7" t="n">
         <v>5026666</v>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>Žedno</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>Donje Testno</t>
         </is>
       </c>
-      <c r="M7" t="n">
+      <c r="N7" t="n">
         <v>12</v>
       </c>
-      <c r="N7" t="n">
+      <c r="O7" t="n">
         <v>4</v>
       </c>
-      <c r="O7" t="n">
+      <c r="P7" t="n">
         <v>200</v>
       </c>
-      <c r="P7" t="inlineStr">
+      <c r="Q7" t="inlineStr">
         <is>
           <t>stari zapis</t>
         </is>
       </c>
-      <c r="Q7" t="inlineStr">
+      <c r="R7" t="inlineStr">
         <is>
           <t>NE</t>
         </is>
       </c>
-      <c r="R7" t="inlineStr">
+      <c r="S7" t="inlineStr">
         <is>
           <t>NE</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr">
+      <c r="T7" t="inlineStr">
         <is>
           <t>NE</t>
         </is>
       </c>
-      <c r="T7" t="inlineStr">
+      <c r="U7" t="inlineStr">
         <is>
           <t>1960</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Jama bez broja</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Renata</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Testni kras</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Testno Selo</t>
+        </is>
+      </c>
+      <c r="O8" t="n">
+        <v>6</v>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>2019</t>
         </is>
       </c>
     </row>

</xml_diff>